<commit_message>
VIES in inglese e cinese, con modello Excel trilingue
- Pagina VIES tradotta: sezioni 1-6, tabelle, avvisi, stati di avanzamento,
  messaggi a comparsa e istruzioni "cosa fare" per ogni riga bloccata.
- Errori e motivi di blocco restano generati e salvati in italiano (dati delle
  pratiche, dei lotti e del controllo finale) e vengono tradotti solo a video;
  un testo senza regola resta in italiano.
- Tipi di documento obbligatori con etichette nelle tre lingue.
- Modello Excel: intestazioni, foglio DATI FOGLIO e istruzioni in italiano,
  inglese e cinese. Il lettore riconosce le colonne in qualunque delle tre
  lingue (anche Excel con intestazioni solo in inglese o solo in cinese) e
  continua a leggere il vecchio modello italiano.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017PtcqmktKbRhYDRcMGmPdu
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -4,129 +4,197 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="PRATICHE" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="DATI FOGLIO" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="ISTRUZIONI" state="visible" r:id="rId6"/>
+    <sheet sheetId="1" name="PRATICHE · APPLICATIONS · 申请" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="DATI FOGLIO · SHEET DATA · 表格信息" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="ISTRUZIONI · INSTRUCTIONS · 说明" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
-  <si>
-    <t>RICHIESTA FIDEIUSSIONI VIES</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+  <si>
+    <t>RICHIESTA FIDEIUSSIONI VIES  ·  VIES GUARANTEE REQUEST  ·  VIES 担保申请</t>
   </si>
   <si>
     <t>Lotto di massimo 20 pratiche · uno ZIP per pratica (1.zip … 20.zip) · beneficiario e rappresentante fiscale nel foglio DATI FOGLIO</t>
   </si>
   <si>
-    <t>ZIP</t>
-  </si>
-  <si>
-    <t>Ragione Sociale</t>
-  </si>
-  <si>
-    <t>Denominazione CN</t>
-  </si>
-  <si>
-    <t>P.IVA</t>
-  </si>
-  <si>
-    <t>Codice credito sociale</t>
-  </si>
-  <si>
-    <t>Sede legale estera</t>
-  </si>
-  <si>
-    <t>Legale rappresentante</t>
-  </si>
-  <si>
-    <t>Documento identità legale rappresentante</t>
-  </si>
-  <si>
-    <t>Data di nascita legale rappresentante</t>
-  </si>
-  <si>
-    <t>Telefono</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>PEC</t>
-  </si>
-  <si>
-    <t>DATI DEL FOGLIO</t>
+    <t>Batch of at most 20 applications · one ZIP per application (1.zip … 20.zip) · beneficiary and fiscal representative in the DATI FOGLIO sheet</t>
+  </si>
+  <si>
+    <t>每批最多 20 笔申请 · 每笔申请一个 ZIP（1.zip … 20.zip）· 受益人和税务代表填写在 DATI FOGLIO 工作表中</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZIP
+ZIP number
+ZIP 编号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ragione Sociale
+Company name
+公司名称</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denominazione CN
+Chinese name
+中文名称</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P.IVA
+Italian VAT number
+意大利增值税号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codice credito sociale
+Unified Social Credit Code
+统一社会信用代码</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sede legale estera
+Registered office abroad
+境外注册地址</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legale rappresentante
+Legal representative
+法定代表人</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento identità legale rappresentante
+Legal representative ID number
+法定代表人身份证号码</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data di nascita legale rappresentante
+Legal representative date of birth
+法定代表人出生日期</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telefono
+Phone
+电话</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Email
+Email
+电子邮箱</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEC
+PEC (certified email)
+PEC 认证邮箱</t>
+  </si>
+  <si>
+    <t>DATI DEL FOGLIO  ·  SHEET DATA  ·  表格信息</t>
   </si>
   <si>
     <t>Beneficiario e rappresentante fiscale validi per tutte le pratiche del lotto</t>
   </si>
   <si>
-    <t>Campo</t>
-  </si>
-  <si>
-    <t>Valore</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>Beneficiario</t>
+    <t>Beneficiary and fiscal representative valid for every application of the batch</t>
+  </si>
+  <si>
+    <t>受益人和税务代表适用于本批次的所有申请</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Campo
+Field
+字段</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valore
+Value
+值</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note
+Notes
+备注</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beneficiario
+Beneficiary
+受益人</t>
   </si>
   <si>
     <t>Agenzia delle Entrate – Direzione Provinciale I di Roma</t>
   </si>
   <si>
-    <t>Ufficio dell'Agenzia competente per il foglio</t>
-  </si>
-  <si>
-    <t>Indirizzo beneficiario</t>
+    <t xml:space="preserve">Ufficio dell'Agenzia competente per il foglio
+Competent office of the Italian Revenue Agency
+主管的意大利税务局办公室</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indirizzo beneficiario
+Beneficiary address
+受益人地址</t>
   </si>
   <si>
     <t>Via Ippolito Nievo, 48 – 00153 Roma (RM)</t>
   </si>
   <si>
-    <t>Indirizzo completo dell'ufficio</t>
-  </si>
-  <si>
-    <t>Codice fiscale beneficiario</t>
+    <t xml:space="preserve">Indirizzo completo dell'ufficio
+Full address of the office
+该办公室的完整地址</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codice fiscale beneficiario
+Beneficiary tax code
+受益人税号</t>
   </si>
   <si>
     <t>06363391001</t>
   </si>
   <si>
-    <t>Codice fiscale dell'Agenzia delle Entrate</t>
-  </si>
-  <si>
-    <t>Rappresentante fiscale</t>
+    <t xml:space="preserve">Codice fiscale dell'Agenzia delle Entrate
+Tax code of the Italian Revenue Agency
+意大利税务局税号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rappresentante fiscale
+Fiscal representative
+税务代表</t>
   </si>
   <si>
     <t>SE&amp;SE AUDITORS &amp; CHARTERED ACCOUNTANT S.P.A. SOCIETA' TRA PROFESSIONISTI</t>
   </si>
   <si>
-    <t>Società di rappresentanza, come da visura</t>
-  </si>
-  <si>
-    <t>Codice fiscale rappresentante fiscale</t>
+    <t xml:space="preserve">Società di rappresentanza, come da visura
+Representative company, as in the registry extract (visura)
+税务代表公司，以商会注册证明为准</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codice fiscale rappresentante fiscale
+Fiscal representative tax code
+税务代表税号</t>
   </si>
   <si>
     <t>13489331002</t>
   </si>
   <si>
-    <t>Codice fiscale / P.IVA della società</t>
-  </si>
-  <si>
-    <t>Amministratore rappresentante fiscale</t>
+    <t xml:space="preserve">Codice fiscale / P.IVA della società
+Company tax code / VAT number
+公司税号 / 增值税号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Amministratore rappresentante fiscale
+Fiscal representative director
+税务代表董事</t>
   </si>
   <si>
     <t>COLCERASA FRANCESCO</t>
   </si>
   <si>
-    <t>Legale rappresentante dalla visura</t>
-  </si>
-  <si>
-    <t>Codice fiscale amministratore</t>
+    <t xml:space="preserve">Legale rappresentante dalla visura
+Legal representative, from the registry extract
+法定代表人，以注册证明为准</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codice fiscale amministratore
+Director tax code
+董事税号</t>
   </si>
   <si>
     <t>CLCFNC61C23H501U</t>
@@ -135,25 +203,36 @@
     <t/>
   </si>
   <si>
-    <t>Sede rappresentante fiscale</t>
+    <t xml:space="preserve">Sede rappresentante fiscale
+Fiscal representative office
+税务代表地址</t>
   </si>
   <si>
     <t>ROMA (RM) VIA DEGLI SCIPIONI 157 CAP 00192</t>
   </si>
   <si>
-    <t>È anche il domicilio fiscale in Italia delle società clienti</t>
-  </si>
-  <si>
-    <t>PEC rappresentante fiscale</t>
+    <t xml:space="preserve">È anche il domicilio fiscale in Italia delle società clienti
+Also the Italian tax domicile of the client companies
+也是客户公司在意大利的税务住所</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEC rappresentante fiscale
+Fiscal representative PEC
+税务代表 PEC</t>
   </si>
   <si>
     <t>servixsrls@pec.it</t>
   </si>
   <si>
-    <t>Usata per i clienti senza PEC propria</t>
-  </si>
-  <si>
-    <t>MODELLO VIES — ISTRUZIONI</t>
+    <t xml:space="preserve">Usata per i clienti senza PEC propria
+Used for clients without their own PEC
+用于没有自己 PEC 的客户</t>
+  </si>
+  <si>
+    <t>MODELLO VIES — ISTRUZIONI  ·  VIES TEMPLATE — INSTRUCTIONS  ·  VIES 模板 — 填写说明</t>
+  </si>
+  <si>
+    <t>ITALIANO</t>
   </si>
   <si>
     <t>1. Un file Excel = un lotto di massimo 20 pratiche.</t>
@@ -193,13 +272,97 @@
   </si>
   <si>
     <t>9. I documenti vengono riconosciuti dal contenuto, non dal nome del file. Una pratica con documenti mancanti o di un'altra società viene bloccata.</t>
+  </si>
+  <si>
+    <t>ENGLISH</t>
+  </si>
+  <si>
+    <t>1. One Excel file = one batch of at most 20 applications.</t>
+  </si>
+  <si>
+    <t>2. PRATICHE sheet: one row per client, starting from row 7. The ZIP column is already numbered 1 to 20: the client on the row with ZIP 3 goes in the file 3.zip.</t>
+  </si>
+  <si>
+    <t>3. Do not change the headers in row 6 and do not insert rows above the table: the portal reads the data from there.</t>
+  </si>
+  <si>
+    <t>4. Rows with only the ZIP number and no other data are ignored.</t>
+  </si>
+  <si>
+    <t>5. The Italian VAT number is optional if the client does not have one yet: the Unified Social Credit Code applies (18 characters, with check character).</t>
+  </si>
+  <si>
+    <t>6. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
+  </si>
+  <si>
+    <t>7. DATI FOGLIO sheet: beneficiary (office of the Italian Revenue Agency) and fiscal representative, the same for the whole batch.</t>
+  </si>
+  <si>
+    <t>8. Each ZIP must contain the documents of the client and of the fiscal representative:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    client: business licence with translation, legal representative's identity document with translation,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    corporate credit report with translation, self-certification supporting the guarantee,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    UBO declaration, fiscal representation mandate;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    fiscal representative: registry extract (visura), financial statements, articles of association.</t>
+  </si>
+  <si>
+    <t>9. Documents are recognised by their content, not by the file name. An application with missing documents, or documents of another company, is blocked.</t>
+  </si>
+  <si>
+    <t>中文</t>
+  </si>
+  <si>
+    <t>1. 一个 Excel 文件 = 一个批次，最多 20 笔申请。</t>
+  </si>
+  <si>
+    <t>2. PRATICHE 工作表：每个客户一行，从第 7 行开始。ZIP 列已编号 1 至 20：ZIP 编号为 3 的那一行客户，其文件放入 3.zip。</t>
+  </si>
+  <si>
+    <t>3. 请勿修改第 6 行的表头，也不要在表格上方插入行：门户从该位置读取数据。</t>
+  </si>
+  <si>
+    <t>4. 只有 ZIP 编号而没有其他数据的行将被忽略。</t>
+  </si>
+  <si>
+    <t>5. 如客户尚无意大利增值税号，可不填写：以统一社会信用代码为准（18 位，含校验位）。</t>
+  </si>
+  <si>
+    <t>6. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>
+  </si>
+  <si>
+    <t>7. DATI FOGLIO 工作表：受益人（意大利税务局办公室）和税务代表，整个批次相同。</t>
+  </si>
+  <si>
+    <t>8. 每个 ZIP 必须包含客户和税务代表的文件：</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    客户：营业执照及翻译件、法定代表人身份证件及翻译件、</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    企业信用信息报告及翻译件、担保所需声明（替代声明）、</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    最终受益人（UBO）声明、税务代表授权书；</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    税务代表：商会注册证明（visura）、财务报表、公司章程。</t>
+  </si>
+  <si>
+    <t>9. 系统按文件内容（而非文件名）识别文件。缺少文件或包含其他公司文件的申请将被阻止。</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -244,6 +407,12 @@
     <font>
       <color rgb="FF667085"/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF103657"/>
+      <sz val="12"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -306,7 +475,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -333,7 +502,7 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -342,7 +511,7 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -350,6 +519,7 @@
     <xf numFmtId="49" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -373,7 +543,7 @@
   <xdr:oneCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>10500</xdr:colOff>
+      <xdr:colOff>16500</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>54000</xdr:rowOff>
     </xdr:from>
@@ -825,72 +995,81 @@
   <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="7" customWidth="1"/>
+    <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="44" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="23" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="60" customWidth="1"/>
-    <col min="7" max="8" width="24" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="26" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="11" width="32" customWidth="1"/>
     <col min="12" max="12" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
     <row r="2" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C2" s="1" t="s">
-        <v>0</v>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
     <row r="5" ht="8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" ht="50" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1216,11 +1395,11 @@
   </sheetData>
   <autoFilter ref="A6:L6"/>
   <dataValidations count="2">
-    <dataValidation type="whole" showErrorMessage="1" errorTitle="Numero ZIP" error="Il numero ZIP va da 1 a 20." sqref="A10:A26">
+    <dataValidation type="whole" showErrorMessage="1" errorTitle="ZIP" error="Il numero ZIP va da 1 a 20. / The ZIP number goes from 1 to 20. / ZIP 编号为 1 至 20。" sqref="A10:A26">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation type="whole" showErrorMessage="1" errorTitle="Numero ZIP" error="Il numero ZIP va da 1 a 20." sqref="A7:A26">
+    <dataValidation type="whole" showErrorMessage="1" errorTitle="ZIP" error="Il numero ZIP va da 1 a 20. / The ZIP number goes from 1 to 20. / ZIP 编号为 1 至 20。" sqref="A7:A26">
       <formula1>1</formula1>
       <formula2>20</formula2>
     </dataValidation>
@@ -1241,131 +1420,139 @@
     <col min="3" max="3" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
     <row r="2" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="1" t="s">
-        <v>14</v>
+      <c r="B2" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="5" ht="8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" ht="32" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" ht="50" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1377,7 +1564,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="150" customWidth="1"/>
@@ -1398,72 +1585,217 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>48</v>
+      <c r="A9" s="18" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
-        <v>49</v>
+      <c r="A10" s="18" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
-        <v>50</v>
+      <c r="A11" s="18" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>51</v>
+      <c r="A12" s="18" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>52</v>
+      <c r="A13" s="18" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
-        <v>53</v>
+      <c r="A14" s="18" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
-        <v>54</v>
+      <c r="A15" s="18" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
-        <v>55</v>
+      <c r="A16" s="18" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
-        <v>56</v>
+      <c r="A17" s="18" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
-        <v>57</v>
+      <c r="A18" s="18" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="17" t="s">
-        <v>58</v>
+      <c r="A19" s="18" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17" t="s">
-        <v>59</v>
+      <c r="A20" s="18" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="17" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="18" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="18" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="18" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="18" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="18" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="18" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="18" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="18" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="18" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="18" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="18" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="18" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="18" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="18" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="18" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="18" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="18" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="18" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
VIES template: no third-party data, fiscal representative block left to fill in
The downloadable template carried the real data of one fiscal representative
(company, administrator and his tax code). It goes to every representative, so
that block is now empty and each note shows an example of the value to enter.
The beneficiary office stays filled in. Instructions updated in the three
languages.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017PtcqmktKbRhYDRcMGmPdu
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>RICHIESTA FIDEIUSSIONI VIES  ·  VIES GUARANTEE REQUEST  ·  VIES 担保申请</t>
   </si>
@@ -191,12 +191,9 @@
 税务代表</t>
   </si>
   <si>
-    <t>SE&amp;SE AUDITORS &amp; CHARTERED ACCOUNTANT S.P.A. SOCIETA' TRA PROFESSIONISTI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Società di rappresentanza, come da visura
-Representative company, as in the registry extract (visura)
-税务代表公司，以商会注册证明为准</t>
+    <t xml:space="preserve">Società di rappresentanza, come da visura. Esempio: ESEMPIO RAPPRESENTANTE FISCALE S.P.A.
+Representative company, as in the registry extract (visura). Example: ESEMPIO RAPPRESENTANTE FISCALE S.P.A.
+税务代表公司，以商会注册证明为准。示例：ESEMPIO RAPPRESENTANTE FISCALE S.P.A.</t>
   </si>
   <si>
     <t xml:space="preserve">Codice fiscale rappresentante fiscale
@@ -204,12 +201,9 @@
 税务代表税号</t>
   </si>
   <si>
-    <t>13489331002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Codice fiscale / P.IVA della società
-Company tax code / VAT number
-公司税号 / 增值税号</t>
+    <t xml:space="preserve">Codice fiscale / P.IVA della società. Esempio: 12345678901
+Company tax code / VAT number. Example: 12345678901
+公司税号 / 增值税号。示例：12345678901</t>
   </si>
   <si>
     <t xml:space="preserve">Amministratore rappresentante fiscale
@@ -217,12 +211,9 @@
 税务代表董事</t>
   </si>
   <si>
-    <t>COLCERASA FRANCESCO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Legale rappresentante dalla visura
-Legal representative, from the registry extract
-法定代表人，以注册证明为准</t>
+    <t xml:space="preserve">Legale rappresentante dalla visura. Esempio: ROSSI MARIO
+Legal representative, from the registry extract. Example: ROSSI MARIO
+法定代表人，以注册证明为准。示例：ROSSI MARIO</t>
   </si>
   <si>
     <t xml:space="preserve">Codice fiscale amministratore
@@ -230,7 +221,9 @@
 董事税号</t>
   </si>
   <si>
-    <t>CLCFNC61C23H501U</t>
+    <t xml:space="preserve">Esempio: RSSMRA70A01H501S
+Example: RSSMRA70A01H501S
+示例：RSSMRA70A01H501S</t>
   </si>
   <si>
     <t xml:space="preserve">Sede rappresentante fiscale
@@ -238,12 +231,9 @@
 税务代表地址</t>
   </si>
   <si>
-    <t>ROMA (RM) VIA DEGLI SCIPIONI 157 CAP 00192</t>
-  </si>
-  <si>
-    <t xml:space="preserve">È anche il domicilio fiscale in Italia delle società clienti
-Also the Italian tax domicile of the client companies
-也是客户公司在意大利的税务住所</t>
+    <t xml:space="preserve">È anche il domicilio fiscale in Italia delle società clienti. Esempio: ROMA (RM) VIA ESEMPIO 1 CAP 00100
+Also the Italian tax domicile of the client companies. Example: ROMA (RM) VIA ESEMPIO 1 CAP 00100
+也是客户公司在意大利的税务住所。示例：ROMA (RM) VIA ESEMPIO 1 CAP 00100</t>
   </si>
   <si>
     <t xml:space="preserve">PEC rappresentante fiscale
@@ -251,12 +241,9 @@
 税务代表 PEC</t>
   </si>
   <si>
-    <t>servixsrls@pec.it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Usata per i clienti senza PEC propria
-Used for clients without their own PEC
-用于没有自己 PEC 的客户</t>
+    <t xml:space="preserve">Usata per i clienti senza PEC propria. Esempio: studio@pec.esempio.it
+Used for clients without their own PEC. Example: studio@pec.esempio.it
+用于没有自己 PEC 的客户。示例：studio@pec.esempio.it</t>
   </si>
   <si>
     <t>MODELLO VIES — ISTRUZIONI  ·  VIES TEMPLATE — INSTRUCTIONS  ·  VIES 模板 — 填写说明</t>
@@ -286,7 +273,7 @@
     <t>7. PEC: lasciare vuota se il cliente non ne ha una: si usa quella del rappresentante fiscale.</t>
   </si>
   <si>
-    <t>8. Foglio DATI FOGLIO: beneficiario (ufficio dell'Agenzia delle Entrate) e rappresentante fiscale, uguali per tutto il lotto. La PEC del beneficiario è facoltativa.</t>
+    <t>8. Foglio DATI FOGLIO: uguale per tutte le pratiche del lotto. Il beneficiario (ufficio dell'Agenzia delle Entrate) è già indicato; la sua PEC è facoltativa. Il rappresentante fiscale va compilato con i vostri dati, come da visura (le note a destra mostrano un esempio per ogni campo).</t>
   </si>
   <si>
     <t>9. Ogni ZIP deve contenere i documenti del cliente e del rappresentante fiscale:</t>
@@ -331,7 +318,7 @@
     <t>7. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
   </si>
   <si>
-    <t>8. DATI FOGLIO sheet: beneficiary (office of the Italian Revenue Agency) and fiscal representative, the same for the whole batch. The beneficiary's PEC is optional.</t>
+    <t>8. DATI FOGLIO sheet: the same for every application of the batch. The beneficiary (office of the Italian Revenue Agency) is already filled in; its PEC is optional. Fill in the fiscal representative with your own data, as in the registry extract (visura): the notes on the right show an example for each field.</t>
   </si>
   <si>
     <t>9. Each ZIP must contain the documents of the client and of the fiscal representative:</t>
@@ -376,7 +363,7 @@
     <t>7. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>
   </si>
   <si>
-    <t>8. DATI FOGLIO 工作表：受益人（意大利税务局办公室）和税务代表，整个批次相同。受益人的 PEC 为可选项。</t>
+    <t>8. DATI FOGLIO 工作表：整个批次的所有申请相同。受益人（意大利税务局办公室）已填写，其 PEC 为可选项。税务代表请按商会注册证明（visura）填写您自己的信息（右侧备注为每个字段提供了示例）。</t>
   </si>
   <si>
     <t>9. 每个 ZIP 必须包含客户和税务代表的文件：</t>
@@ -1541,64 +1528,54 @@
       <c r="A11" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="15"/>
+      <c r="C11" s="16" t="s">
         <v>44</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>50</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="C14" s="19"/>
+        <v>49</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="19" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B15" s="15" t="s">
-        <v>55</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="B15" s="15"/>
       <c r="C15" s="16" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="B16" s="18" t="s">
-        <v>58</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="B16" s="18"/>
       <c r="C16" s="19" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1631,232 +1608,232 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" s="21" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="21" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="21" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="21" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
MUP unico su carta intestata al posto di privacy/MUP/antiriciclaggio; nuove colonne dell'Excel del lotto (con ID del rappresentante fiscale)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGdYVAKxyB91ytB8iWpM65
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
   <si>
     <t>RICHIESTA FIDEIUSSIONI VIES  ·  VIES GUARANTEE REQUEST  ·  VIES 担保申请</t>
   </si>
@@ -32,14 +32,29 @@
 ZIP 编号</t>
   </si>
   <si>
+    <t xml:space="preserve">ID
+ID
+编号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo Anagrafica
+Entity type
+主体类型</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ragione Sociale
 Company name
 公司名称</t>
   </si>
   <si>
-    <t xml:space="preserve">Denominazione CN
-Chinese name
-中文名称</t>
+    <t xml:space="preserve">Tipo Società
+Company type
+公司类型</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C.F.
+Tax code
+税号</t>
   </si>
   <si>
     <t xml:space="preserve">P.IVA
@@ -47,29 +62,44 @@
 意大利增值税号</t>
   </si>
   <si>
-    <t xml:space="preserve">Codice credito sociale
-Unified Social Credit Code
-统一社会信用代码</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sede legale estera
-Registered office abroad
-境外注册地址</t>
-  </si>
-  <si>
     <t xml:space="preserve">Legale rappresentante
 Legal representative
 法定代表人</t>
   </si>
   <si>
-    <t xml:space="preserve">Telefono
-Phone
-电话</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Email
-Email
-电子邮箱</t>
+    <t xml:space="preserve">Indirizzo (via, piazza…)
+Address (street, square…)
+地址（街道、广场…）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Numero civico
+Street number
+门牌号</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Città
+City
+城市</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAP
+Postal code
+邮编</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia
+Province
+省份</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nazione
+Country
+国家</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sede principale
+Main office
+主要办事处</t>
   </si>
   <si>
     <t xml:space="preserve">PEC
@@ -77,31 +107,52 @@
 PEC 认证邮箱</t>
   </si>
   <si>
+    <t>RF-0001</t>
+  </si>
+  <si>
+    <t>persona giuridica</t>
+  </si>
+  <si>
     <t>ESEMPIO · completo · SAMPLE TRADING CO.</t>
   </si>
   <si>
-    <t>示例贸易有限公司</t>
+    <t>srl</t>
+  </si>
+  <si>
+    <t>91440300EXAMPLE001</t>
   </si>
   <si>
     <t>01234567890</t>
   </si>
   <si>
-    <t>91440300EXAMPLE001</t>
-  </si>
-  <si>
-    <t>Room 101, Building 1, Sample Road 1, Nanshan District, Shenzhen, China</t>
-  </si>
-  <si>
     <t>ZHANG WEI</t>
   </si>
   <si>
-    <t>+86 755 0000 0000</t>
-  </si>
-  <si>
-    <t>nome@esempio.com</t>
+    <t>Via Esempio</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Milano</t>
+  </si>
+  <si>
+    <t>20100</t>
+  </si>
+  <si>
+    <t>MI</t>
+  </si>
+  <si>
+    <t>Italia</t>
+  </si>
+  <si>
+    <t>Sì</t>
   </si>
   <si>
     <t>societa@pec.esempio.it</t>
+  </si>
+  <si>
+    <t>RF-0002</t>
   </si>
   <si>
     <t>ESEMPIO · solo obbligatori · MINIMUM DATA CO.</t>
@@ -267,16 +318,22 @@
     <t>5. Le righe con solo il numero ZIP e nessun altro dato vengono ignorate.</t>
   </si>
   <si>
-    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e almeno uno tra P.IVA e Codice credito sociale (18 caratteri, con cifra di controllo). Tutte le altre colonne sono facoltative.</t>
-  </si>
-  <si>
-    <t>7. PEC: lasciare vuota se il cliente non ne ha una: si usa quella del rappresentante fiscale.</t>
-  </si>
-  <si>
-    <t>8. Foglio DATI FOGLIO: uguale per tutte le pratiche del lotto. Il beneficiario (ufficio dell'Agenzia delle Entrate) è già indicato; la sua PEC è facoltativa. Il rappresentante fiscale va compilato con i vostri dati, come da visura (le note a destra mostrano un esempio per ogni campo).</t>
-  </si>
-  <si>
-    <t>9. Ogni ZIP deve contenere i documenti del cliente e del rappresentante fiscale:</t>
+    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e almeno uno tra C.F. e P.IVA (il C.F. di una società cinese è il codice di credito sociale, 18 caratteri con cifra di controllo). Tutte le altre colonne sono facoltative.</t>
+  </si>
+  <si>
+    <t>7. ID: il numero interno con cui il rappresentante fiscale ritrova la pratica nel proprio portale (serve solo a voi).</t>
+  </si>
+  <si>
+    <t>8. Tipo Anagrafica (es. persona giuridica), Tipo Società (srl, snc, nessuna), Indirizzo, Numero civico, Città, CAP, Provincia, Nazione e Sede principale (Sì/No) descrivono la sede del cliente.</t>
+  </si>
+  <si>
+    <t>9. PEC: lasciare vuota se il cliente non ne ha una: si usa quella del rappresentante fiscale.</t>
+  </si>
+  <si>
+    <t>10. Foglio DATI FOGLIO: uguale per tutte le pratiche del lotto. Il beneficiario (ufficio dell'Agenzia delle Entrate) è già indicato; la sua PEC è facoltativa. Il rappresentante fiscale va compilato con i vostri dati, come da visura (le note a destra mostrano un esempio per ogni campo).</t>
+  </si>
+  <si>
+    <t>11. Ogni ZIP deve contenere i documenti del cliente e del rappresentante fiscale:</t>
   </si>
   <si>
     <t xml:space="preserve">    cliente: licenza commerciale con traduzione, documento d'identità del legale rappresentante con traduzione,</t>
@@ -291,7 +348,7 @@
     <t xml:space="preserve">    rappresentante fiscale: visura, bilancio, statuto.</t>
   </si>
   <si>
-    <t>10. I documenti vengono riconosciuti dal contenuto, non dal nome del file. Una pratica con documenti mancanti o di un'altra società viene bloccata.</t>
+    <t>12. I documenti vengono riconosciuti dal contenuto, non dal nome del file. Una pratica con documenti mancanti o di un'altra società viene bloccata.</t>
   </si>
   <si>
     <t>ENGLISH</t>
@@ -312,16 +369,22 @@
     <t>5. Rows with only the ZIP number and no other data are ignored.</t>
   </si>
   <si>
-    <t>6. Required for each client: ZIP number, company name and at least one of the Italian VAT number and the Unified Social Credit Code (18 characters, with check character). All other columns are optional.</t>
-  </si>
-  <si>
-    <t>7. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
-  </si>
-  <si>
-    <t>8. DATI FOGLIO sheet: the same for every application of the batch. The beneficiary (office of the Italian Revenue Agency) is already filled in; its PEC is optional. Fill in the fiscal representative with your own data, as in the registry extract (visura): the notes on the right show an example for each field.</t>
-  </si>
-  <si>
-    <t>9. Each ZIP must contain the documents of the client and of the fiscal representative:</t>
+    <t>6. Required for each client: ZIP number, company name and at least one of the tax code and the Italian VAT number (the tax code of a Chinese company is its Unified Social Credit Code, 18 characters with check character). All other columns are optional.</t>
+  </si>
+  <si>
+    <t>7. ID: the internal number the fiscal representative uses to find the practice in their own portal (only for your own use).</t>
+  </si>
+  <si>
+    <t>8. Entity type (e.g. persona giuridica), Company type (srl, snc, nessuna), Address, Street number, City, Postal code, Province, Country and Main office (Yes/No) describe the client's office.</t>
+  </si>
+  <si>
+    <t>9. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
+  </si>
+  <si>
+    <t>10. DATI FOGLIO sheet: the same for every application of the batch. The beneficiary (office of the Italian Revenue Agency) is already filled in; its PEC is optional. Fill in the fiscal representative with your own data, as in the registry extract (visura): the notes on the right show an example for each field.</t>
+  </si>
+  <si>
+    <t>11. Each ZIP must contain the documents of the client and of the fiscal representative:</t>
   </si>
   <si>
     <t xml:space="preserve">    client: business licence with translation, legal representative's identity document with translation,</t>
@@ -336,7 +399,7 @@
     <t xml:space="preserve">    fiscal representative: registry extract (visura), financial statements, articles of association.</t>
   </si>
   <si>
-    <t>10. Documents are recognised by their content, not by the file name. An application with missing documents, or documents of another company, is blocked.</t>
+    <t>12. Documents are recognised by their content, not by the file name. An application with missing documents, or documents of another company, is blocked.</t>
   </si>
   <si>
     <t>中文</t>
@@ -357,16 +420,22 @@
     <t>5. 只有 ZIP 编号而没有其他数据的行将被忽略。</t>
   </si>
   <si>
-    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及意大利增值税号和统一社会信用代码（18 位，含校验位）中的至少一项。其他列均为可选。</t>
-  </si>
-  <si>
-    <t>7. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>
-  </si>
-  <si>
-    <t>8. DATI FOGLIO 工作表：整个批次的所有申请相同。受益人（意大利税务局办公室）已填写，其 PEC 为可选项。税务代表请按商会注册证明（visura）填写您自己的信息（右侧备注为每个字段提供了示例）。</t>
-  </si>
-  <si>
-    <t>9. 每个 ZIP 必须包含客户和税务代表的文件：</t>
+    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及税号和意大利增值税号中的至少一项（中国公司的税号即统一社会信用代码，18 位，含校验位）。其他列均为可选。</t>
+  </si>
+  <si>
+    <t>7. ID：税务代表在其自己的门户中查找该申请所用的内部编号（仅供贵方内部使用）。</t>
+  </si>
+  <si>
+    <t>8. 主体类型（如 persona giuridica）、公司类型（srl、snc、nessuna）、地址、门牌号、城市、邮编、省份、国家和主要办事处（是/否）说明客户的办公地点。</t>
+  </si>
+  <si>
+    <t>9. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>
+  </si>
+  <si>
+    <t>10. DATI FOGLIO 工作表：整个批次的所有申请相同。受益人（意大利税务局办公室）已填写，其 PEC 为可选项。税务代表请按商会注册证明（visura）填写您自己的信息（右侧备注为每个字段提供了示例）。</t>
+  </si>
+  <si>
+    <t>11. 每个 ZIP 必须包含客户和税务代表的文件：</t>
   </si>
   <si>
     <t xml:space="preserve">    客户：营业执照及翻译件、法定代表人身份证件及翻译件、</t>
@@ -381,7 +450,7 @@
     <t xml:space="preserve">    税务代表：商会注册证明（visura）、财务报表、公司章程。</t>
   </si>
   <si>
-    <t>10. 系统按文件内容（而非文件名）识别文件。缺少文件或包含其他公司文件的申请将被阻止。</t>
+    <t>12. 系统按文件内容（而非文件名）识别文件。缺少文件或包含其他公司文件的申请将被阻止。</t>
   </si>
 </sst>
 </file>
@@ -529,28 +598,28 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1044,19 +1113,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:P26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
-    <col min="2" max="2" width="44" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="60" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
-    <col min="8" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="44" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
+    <col min="9" max="9" width="34" customWidth="1"/>
+    <col min="10" max="10" width="12" customWidth="1"/>
+    <col min="11" max="11" width="20" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="16" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="16" max="16" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
@@ -1084,7 +1159,7 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" ht="50" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>4</v>
       </c>
@@ -1115,311 +1190,463 @@
       <c r="J6" s="4" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="L6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="P6" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>1</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>15</v>
+        <v>20</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>27</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="6"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F8" s="6"/>
+        <v>35</v>
+      </c>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="7"/>
+      <c r="F8" s="6" t="s">
+        <v>37</v>
+      </c>
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="6"/>
+      <c r="I8" s="7"/>
       <c r="J8" s="6"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K8" s="7"/>
+      <c r="L8" s="6"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
+      <c r="O8" s="7"/>
+      <c r="P8" s="7"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>3</v>
       </c>
       <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
+      <c r="C9" s="10"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="10"/>
-      <c r="I9" s="9"/>
+      <c r="I9" s="10"/>
       <c r="J9" s="9"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K9" s="10"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
         <v>4</v>
       </c>
       <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
+      <c r="C10" s="13"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="13"/>
-      <c r="I10" s="12"/>
+      <c r="I10" s="13"/>
       <c r="J10" s="12"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K10" s="13"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>5</v>
       </c>
       <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
+      <c r="C11" s="10"/>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="9"/>
       <c r="G11" s="9"/>
       <c r="H11" s="10"/>
-      <c r="I11" s="9"/>
+      <c r="I11" s="10"/>
       <c r="J11" s="9"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K11" s="10"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="10"/>
+      <c r="N11" s="10"/>
+      <c r="O11" s="10"/>
+      <c r="P11" s="10"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
         <v>6</v>
       </c>
       <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
+      <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="12"/>
       <c r="G12" s="12"/>
       <c r="H12" s="13"/>
-      <c r="I12" s="12"/>
+      <c r="I12" s="13"/>
       <c r="J12" s="12"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K12" s="13"/>
+      <c r="L12" s="12"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>7</v>
       </c>
       <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
+      <c r="C13" s="10"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="9"/>
       <c r="G13" s="9"/>
       <c r="H13" s="10"/>
-      <c r="I13" s="9"/>
+      <c r="I13" s="10"/>
       <c r="J13" s="9"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K13" s="10"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="10"/>
+      <c r="N13" s="10"/>
+      <c r="O13" s="10"/>
+      <c r="P13" s="10"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
         <v>8</v>
       </c>
       <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
+      <c r="C14" s="13"/>
       <c r="D14" s="13"/>
       <c r="E14" s="13"/>
       <c r="F14" s="12"/>
       <c r="G14" s="12"/>
       <c r="H14" s="13"/>
-      <c r="I14" s="12"/>
+      <c r="I14" s="13"/>
       <c r="J14" s="12"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K14" s="13"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>9</v>
       </c>
       <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
+      <c r="C15" s="10"/>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
       <c r="F15" s="9"/>
       <c r="G15" s="9"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="9"/>
+      <c r="I15" s="10"/>
       <c r="J15" s="9"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K15" s="10"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="10"/>
+      <c r="N15" s="10"/>
+      <c r="O15" s="10"/>
+      <c r="P15" s="10"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
         <v>10</v>
       </c>
       <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
+      <c r="C16" s="13"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="12"/>
       <c r="G16" s="12"/>
       <c r="H16" s="13"/>
-      <c r="I16" s="12"/>
+      <c r="I16" s="13"/>
       <c r="J16" s="12"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K16" s="13"/>
+      <c r="L16" s="12"/>
+      <c r="M16" s="13"/>
+      <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
+      <c r="P16" s="13"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>11</v>
       </c>
       <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
+      <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="9"/>
+      <c r="I17" s="10"/>
       <c r="J17" s="9"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K17" s="10"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="10"/>
+      <c r="N17" s="10"/>
+      <c r="O17" s="10"/>
+      <c r="P17" s="10"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
         <v>12</v>
       </c>
       <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
+      <c r="C18" s="13"/>
       <c r="D18" s="13"/>
       <c r="E18" s="13"/>
       <c r="F18" s="12"/>
       <c r="G18" s="12"/>
       <c r="H18" s="13"/>
-      <c r="I18" s="12"/>
+      <c r="I18" s="13"/>
       <c r="J18" s="12"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K18" s="13"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>13</v>
       </c>
       <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
+      <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="9"/>
       <c r="G19" s="9"/>
       <c r="H19" s="10"/>
-      <c r="I19" s="9"/>
+      <c r="I19" s="10"/>
       <c r="J19" s="9"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K19" s="10"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="10"/>
+      <c r="N19" s="10"/>
+      <c r="O19" s="10"/>
+      <c r="P19" s="10"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
         <v>14</v>
       </c>
       <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
+      <c r="C20" s="13"/>
       <c r="D20" s="13"/>
       <c r="E20" s="13"/>
       <c r="F20" s="12"/>
       <c r="G20" s="12"/>
       <c r="H20" s="13"/>
-      <c r="I20" s="12"/>
+      <c r="I20" s="13"/>
       <c r="J20" s="12"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K20" s="13"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>15</v>
       </c>
       <c r="B21" s="9"/>
-      <c r="C21" s="9"/>
+      <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="9"/>
       <c r="G21" s="9"/>
       <c r="H21" s="10"/>
-      <c r="I21" s="9"/>
+      <c r="I21" s="10"/>
       <c r="J21" s="9"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K21" s="10"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="10"/>
+      <c r="N21" s="10"/>
+      <c r="O21" s="10"/>
+      <c r="P21" s="10"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
         <v>16</v>
       </c>
       <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
+      <c r="C22" s="13"/>
       <c r="D22" s="13"/>
       <c r="E22" s="13"/>
       <c r="F22" s="12"/>
       <c r="G22" s="12"/>
       <c r="H22" s="13"/>
-      <c r="I22" s="12"/>
+      <c r="I22" s="13"/>
       <c r="J22" s="12"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K22" s="13"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>17</v>
       </c>
       <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
+      <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="9"/>
       <c r="G23" s="9"/>
       <c r="H23" s="10"/>
-      <c r="I23" s="9"/>
+      <c r="I23" s="10"/>
       <c r="J23" s="9"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K23" s="10"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="10"/>
+      <c r="N23" s="10"/>
+      <c r="O23" s="10"/>
+      <c r="P23" s="10"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="11">
         <v>18</v>
       </c>
       <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
+      <c r="C24" s="13"/>
       <c r="D24" s="13"/>
       <c r="E24" s="13"/>
       <c r="F24" s="12"/>
       <c r="G24" s="12"/>
       <c r="H24" s="13"/>
-      <c r="I24" s="12"/>
+      <c r="I24" s="13"/>
       <c r="J24" s="12"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K24" s="13"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" s="8">
         <v>19</v>
       </c>
       <c r="B25" s="9"/>
-      <c r="C25" s="9"/>
+      <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="10"/>
-      <c r="I25" s="9"/>
+      <c r="I25" s="10"/>
       <c r="J25" s="9"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K25" s="10"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="10"/>
+      <c r="N25" s="10"/>
+      <c r="O25" s="10"/>
+      <c r="P25" s="10"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
         <v>20</v>
       </c>
       <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
+      <c r="C26" s="13"/>
       <c r="D26" s="13"/>
       <c r="E26" s="13"/>
       <c r="F26" s="12"/>
       <c r="G26" s="12"/>
       <c r="H26" s="13"/>
-      <c r="I26" s="12"/>
+      <c r="I26" s="13"/>
       <c r="J26" s="12"/>
+      <c r="K26" s="13"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
     </row>
   </sheetData>
-  <autoFilter ref="A6:J6"/>
+  <autoFilter ref="A6:P6"/>
   <dataValidations count="2">
     <dataValidation type="whole" showErrorMessage="1" errorTitle="ZIP" error="Il numero ZIP va da 1 a 20. / The ZIP number goes from 1 to 20. / ZIP 编号为 1 至 20。" sqref="A10:A26">
       <formula1>1</formula1>
@@ -1448,22 +1675,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1473,109 +1700,109 @@
     </row>
     <row r="6" ht="50" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C8" s="19" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="19" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="16" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="19" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="19" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="16" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="19" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1587,7 +1814,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="150" customWidth="1"/>
@@ -1608,232 +1835,262 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>70</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="21" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="20" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="21" t="s">
-        <v>72</v>
+      <c r="A24" s="21" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="21" t="s">
-        <v>73</v>
+      <c r="A26" s="20" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>85</v>
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="21" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" s="20" t="s">
-        <v>86</v>
+      <c r="A40" s="21" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" s="21" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" s="21" t="s">
-        <v>90</v>
+      <c r="A44" s="20" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
-        <v>100</v>
+        <v>113</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="21" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="21" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="21" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="21" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="21" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="21" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel del lotto: C.F. della società cinese (Agenzia delle Entrate), indirizzo scomposto sulla pratica, Sede principale da compilare
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGdYVAKxyB91ytB8iWpM65
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="118">
   <si>
     <t>RICHIESTA FIDEIUSSIONI VIES  ·  VIES GUARANTEE REQUEST  ·  VIES 担保申请</t>
   </si>
@@ -119,7 +119,7 @@
     <t>srl</t>
   </si>
   <si>
-    <t>91440300EXAMPLE001</t>
+    <t>98765432109</t>
   </si>
   <si>
     <t>01234567890</t>
@@ -146,9 +146,6 @@
     <t>Italia</t>
   </si>
   <si>
-    <t>Sì</t>
-  </si>
-  <si>
     <t>societa@pec.esempio.it</t>
   </si>
   <si>
@@ -156,9 +153,6 @@
   </si>
   <si>
     <t>ESEMPIO · solo obbligatori · MINIMUM DATA CO.</t>
-  </si>
-  <si>
-    <t>91310000EXAMPLE002</t>
   </si>
   <si>
     <t>DATI DEL FOGLIO  ·  SHEET DATA  ·  表格信息</t>
@@ -318,13 +312,13 @@
     <t>5. Le righe con solo il numero ZIP e nessun altro dato vengono ignorate.</t>
   </si>
   <si>
-    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e almeno uno tra C.F. e P.IVA (il C.F. di una società cinese è il codice di credito sociale, 18 caratteri con cifra di controllo). Tutte le altre colonne sono facoltative.</t>
+    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e almeno uno tra C.F. e P.IVA (il C.F. della società cinese è quello assegnato dall'Agenzia delle Entrate insieme alla partita IVA, come nel certificato di attribuzione). Tutte le altre colonne sono facoltative.</t>
   </si>
   <si>
     <t>7. ID: il numero interno con cui il rappresentante fiscale ritrova la pratica nel proprio portale (serve solo a voi).</t>
   </si>
   <si>
-    <t>8. Tipo Anagrafica (es. persona giuridica), Tipo Società (srl, snc, nessuna), Indirizzo, Numero civico, Città, CAP, Provincia, Nazione e Sede principale (Sì/No) descrivono la sede del cliente.</t>
+    <t>8. Tipo Anagrafica (es. persona giuridica), Tipo Società (srl, snc, nessuna), Indirizzo, Numero civico, Città, CAP, Provincia, Nazione e Sede principale descrivono la sede del cliente (da compilare).</t>
   </si>
   <si>
     <t>9. PEC: lasciare vuota se il cliente non ne ha una: si usa quella del rappresentante fiscale.</t>
@@ -369,13 +363,13 @@
     <t>5. Rows with only the ZIP number and no other data are ignored.</t>
   </si>
   <si>
-    <t>6. Required for each client: ZIP number, company name and at least one of the tax code and the Italian VAT number (the tax code of a Chinese company is its Unified Social Credit Code, 18 characters with check character). All other columns are optional.</t>
+    <t>6. Required for each client: ZIP number, company name and at least one of the tax code and the Italian VAT number (the tax code of the Chinese company is the one the Italian Revenue Agency assigned together with the VAT number, as in the attribution certificate). All other columns are optional.</t>
   </si>
   <si>
     <t>7. ID: the internal number the fiscal representative uses to find the practice in their own portal (only for your own use).</t>
   </si>
   <si>
-    <t>8. Entity type (e.g. persona giuridica), Company type (srl, snc, nessuna), Address, Street number, City, Postal code, Province, Country and Main office (Yes/No) describe the client's office.</t>
+    <t>8. Entity type (e.g. persona giuridica), Company type (srl, snc, nessuna), Address, Street number, City, Postal code, Province, Country and Main office describe the client's office (to be filled in).</t>
   </si>
   <si>
     <t>9. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
@@ -420,13 +414,13 @@
     <t>5. 只有 ZIP 编号而没有其他数据的行将被忽略。</t>
   </si>
   <si>
-    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及税号和意大利增值税号中的至少一项（中国公司的税号即统一社会信用代码，18 位，含校验位）。其他列均为可选。</t>
+    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及税号和意大利增值税号中的至少一项（中国公司的税号是意大利税务局与增值税号一并分配的税号，见分配证明）。其他列均为可选。</t>
   </si>
   <si>
     <t>7. ID：税务代表在其自己的门户中查找该申请所用的内部编号（仅供贵方内部使用）。</t>
   </si>
   <si>
-    <t>8. 主体类型（如 persona giuridica）、公司类型（srl、snc、nessuna）、地址、门牌号、城市、邮编、省份、国家和主要办事处（是/否）说明客户的办公地点。</t>
+    <t>8. 主体类型（如 persona giuridica）、公司类型（srl、snc、nessuna）、地址、门牌号、城市、邮编、省份、国家和主要办事处说明客户的办公地点（请填写）。</t>
   </si>
   <si>
     <t>9. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>
@@ -1121,7 +1115,7 @@
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="44" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
     <col min="7" max="7" width="17" customWidth="1"/>
     <col min="8" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="34" customWidth="1"/>
@@ -1252,11 +1246,9 @@
       <c r="N7" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="7"/>
+      <c r="P7" s="7" t="s">
         <v>33</v>
-      </c>
-      <c r="P7" s="7" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1264,15 +1256,15 @@
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" s="7"/>
       <c r="F8" s="6" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="7"/>
@@ -1675,22 +1667,22 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" ht="8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1700,109 +1692,109 @@
     </row>
     <row r="6" ht="50" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>42</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="16" t="s">
         <v>45</v>
-      </c>
-      <c r="B7" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" s="19" t="s">
         <v>48</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>51</v>
-      </c>
-      <c r="B9" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="10" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B10" s="18"/>
       <c r="C10" s="19" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B11" s="15"/>
       <c r="C11" s="16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B12" s="18"/>
       <c r="C12" s="19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B13" s="15"/>
       <c r="C13" s="16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B14" s="18"/>
       <c r="C14" s="19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -1835,262 +1827,262 @@
     </row>
     <row r="6" ht="32" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="21" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" s="21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="21" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" s="21" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" s="21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" s="21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" s="21" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" s="21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="21" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="21" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" s="21" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" s="21" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="21" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" s="21" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" s="21" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" s="21" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="21" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="21" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="21" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="21" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" s="21" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" s="21" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" s="21" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" s="21" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" s="21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" s="21" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" s="21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" s="21" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" s="20" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" s="21" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" s="21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" s="21" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" s="21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="21" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" s="21" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" s="21" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" s="21" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" s="21" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" s="21" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" s="21" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" s="21" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" s="21" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" s="21" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" s="21" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel del lotto: il contraente cinese si identifica solo con la partita IVA italiana, mai con il codice di credito sociale
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGdYVAKxyB91ytB8iWpM65
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -312,7 +312,7 @@
     <t>5. Le righe con solo il numero ZIP e nessun altro dato vengono ignorate.</t>
   </si>
   <si>
-    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e almeno uno tra C.F. e P.IVA (il C.F. della società cinese è quello assegnato dall'Agenzia delle Entrate insieme alla partita IVA, come nel certificato di attribuzione). Tutte le altre colonne sono facoltative.</t>
+    <t>6. Obbligatori per ogni cliente: numero ZIP, Ragione Sociale e la partita IVA italiana assegnata alla società cinese dall'Agenzia delle Entrate (certificato di attribuzione), in P.IVA o in C.F. (è lo stesso numero). Non inserire mai il codice di credito sociale cinese. Tutte le altre colonne sono facoltative.</t>
   </si>
   <si>
     <t>7. ID: il numero interno con cui il rappresentante fiscale ritrova la pratica nel proprio portale (serve solo a voi).</t>
@@ -363,7 +363,7 @@
     <t>5. Rows with only the ZIP number and no other data are ignored.</t>
   </si>
   <si>
-    <t>6. Required for each client: ZIP number, company name and at least one of the tax code and the Italian VAT number (the tax code of the Chinese company is the one the Italian Revenue Agency assigned together with the VAT number, as in the attribution certificate). All other columns are optional.</t>
+    <t>6. Required for each client: ZIP number, company name and the Italian VAT number the Italian Revenue Agency assigned to the Chinese company (attribution certificate), in P.IVA or in C.F. (it is the same number). Never enter the Chinese Unified Social Credit Code. All other columns are optional.</t>
   </si>
   <si>
     <t>7. ID: the internal number the fiscal representative uses to find the practice in their own portal (only for your own use).</t>
@@ -414,7 +414,7 @@
     <t>5. 只有 ZIP 编号而没有其他数据的行将被忽略。</t>
   </si>
   <si>
-    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及税号和意大利增值税号中的至少一项（中国公司的税号是意大利税务局与增值税号一并分配的税号，见分配证明）。其他列均为可选。</t>
+    <t>6. 每个客户的必填项：ZIP 编号、公司名称，以及意大利税务局分配给中国公司的意大利增值税号（见分配证明），填写在 P.IVA 或 C.F. 中（两者为同一号码）。切勿填写中国统一社会信用代码。其他列均为可选。</t>
   </si>
   <si>
     <t>7. ID：税务代表在其自己的门户中查找该申请所用的内部编号（仅供贵方内部使用）。</t>

</xml_diff>

<commit_message>
Excel del lotto: la sede del contraente e' quella del rappresentante fiscale in Italia (istruzioni, guida, etichette)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGdYVAKxyB91ytB8iWpM65
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -318,7 +318,7 @@
     <t>7. ID: il numero interno con cui il rappresentante fiscale ritrova la pratica nel proprio portale (serve solo a voi).</t>
   </si>
   <si>
-    <t>8. Tipo Anagrafica (es. persona giuridica), Tipo Società (srl, snc, nessuna), Indirizzo, Numero civico, Città, CAP, Provincia, Nazione e Sede principale descrivono la sede del cliente (da compilare).</t>
+    <t>8. Tipo Anagrafica (es. persona giuridica), Tipo Società (srl, snc, nessuna), Indirizzo, Numero civico, Città, CAP, Provincia, Nazione e Sede principale descrivono la sede del cliente in Italia, che è quella del rappresentante fiscale (non la sede in Cina); la Sede principale è da compilare.</t>
   </si>
   <si>
     <t>9. PEC: lasciare vuota se il cliente non ne ha una: si usa quella del rappresentante fiscale.</t>
@@ -369,7 +369,7 @@
     <t>7. ID: the internal number the fiscal representative uses to find the practice in their own portal (only for your own use).</t>
   </si>
   <si>
-    <t>8. Entity type (e.g. persona giuridica), Company type (srl, snc, nessuna), Address, Street number, City, Postal code, Province, Country and Main office describe the client's office (to be filled in).</t>
+    <t>8. Entity type (e.g. persona giuridica), Company type (srl, snc, nessuna), Address, Street number, City, Postal code, Province, Country and Main office describe the client's office in Italy, which is the fiscal representative's (not the office in China); Main office is to be filled in.</t>
   </si>
   <si>
     <t>9. PEC: leave it empty if the client has none: the fiscal representative's PEC is used.</t>
@@ -420,7 +420,7 @@
     <t>7. ID：税务代表在其自己的门户中查找该申请所用的内部编号（仅供贵方内部使用）。</t>
   </si>
   <si>
-    <t>8. 主体类型（如 persona giuridica）、公司类型（srl、snc、nessuna）、地址、门牌号、城市、邮编、省份、国家和主要办事处说明客户的办公地点（请填写）。</t>
+    <t>8. 主体类型（如 persona giuridica）、公司类型（srl、snc、nessuna）、地址、门牌号、城市、邮编、省份、国家和主要办事处说明客户在意大利的办公地址，即税务代表的地址（不是中国的地址）；主要办事处请填写。</t>
   </si>
   <si>
     <t>9. PEC：如客户没有 PEC，请留空：将使用税务代表的 PEC。</t>

</xml_diff>

<commit_message>
Modello Excel del lotto con logo e intestazione Tecno Advance MGA
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CGdYVAKxyB91ytB8iWpM65
</commit_message>
<xml_diff>
--- a/public/vies/VIES_modello.xlsx
+++ b/public/vies/VIES_modello.xlsx
@@ -16,7 +16,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="59">
+  <si>
+    <t>RICHIESTA FIDEIUSSIONI VIES  ·  VIES GUARANTEE REQUEST  ·  VIES 担保申请</t>
+  </si>
+  <si>
+    <t>Lotto di massimo 20 pratiche · una riga per cliente · uno ZIP per pratica (1.zip … 20.zip)</t>
+  </si>
   <si>
     <t>ZIP</t>
   </si>
@@ -124,6 +130,12 @@
   </si>
   <si>
     <t>pearlbeauty@pec.example.it</t>
+  </si>
+  <si>
+    <t>RAPPRESENTANTE FISCALE  ·  FISCAL REPRESENTATIVE  ·  税务代表</t>
+  </si>
+  <si>
+    <t>Dati del rappresentante fiscale, validi per tutte le pratiche del lotto</t>
   </si>
   <si>
     <t xml:space="preserve">SE&amp;SE AUDITORS &amp;
@@ -154,6 +166,12 @@
   </si>
   <si>
     <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>BENEFICIARIO  ·  BENEFICIARY  ·  受益人</t>
+  </si>
+  <si>
+    <t>Beneficiario della garanzia, valido per tutte le pratiche del lotto</t>
   </si>
   <si>
     <t>AGENZIA DELLE ENTRATE</t>
@@ -184,12 +202,23 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
       <scheme val="minor"/>
       <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF103657"/>
+      <sz val="16"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <color rgb="FF667085"/>
+      <sz val="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -231,12 +260,21 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFAC7E59"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -265,25 +303,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -301,6 +342,138 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>12000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1828800" cy="666750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>27000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1828800" cy="666750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>27000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>54000</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1828800" cy="666750"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -566,7 +739,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O12"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" defaultColWidth="8.81640625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -576,338 +749,368 @@
     <col min="9" max="15" width="16.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="20" customHeight="1" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="4:4" x14ac:dyDescent="0.25">
+      <c r="D3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+    </row>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="8" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="F6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="G6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="I6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="K6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="M6" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="N6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="O6" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2" t="s">
+      <c r="B7" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="D7" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="E7" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="F7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="H7" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="I7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="L2" s="2" t="s">
+      <c r="J7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="M2" s="2" t="s">
+      <c r="K7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="L7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="M7" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="N7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="2" t="s">
+      <c r="B8" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="O8" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>3</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="2" t="s">
+      <c r="C9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="I9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="J9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="K9" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="L9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="O4" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
-      <c r="L6" s="6"/>
-      <c r="M6" s="6"/>
-      <c r="N6" s="6"/>
-      <c r="O6" s="6"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="6"/>
-      <c r="N7" s="6"/>
-      <c r="O7" s="6"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="6"/>
-      <c r="M8" s="6"/>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="6"/>
-      <c r="M9" s="6"/>
-      <c r="N9" s="6"/>
-      <c r="O9" s="6"/>
+      <c r="M9" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="O9" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
-      <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
-      <c r="O10" s="6"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
+      <c r="N10" s="7"/>
+      <c r="O10" s="7"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="6"/>
-      <c r="M11" s="6"/>
-      <c r="N11" s="6"/>
-      <c r="O11" s="6"/>
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="6"/>
-      <c r="M12" s="6"/>
-      <c r="N12" s="6"/>
-      <c r="O12" s="6"/>
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -926,120 +1129,149 @@
     <col min="14" max="14" width="25.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="8" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="F6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="G6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="I6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="K6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" ht="58" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="M6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="G2" s="2" t="s">
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" ht="58" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="C7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="D7" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="E7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="J7" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="L7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H8" s="8"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="14.5" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1058,111 +1290,140 @@
     <col min="14" max="14" width="44" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
+    <row r="1" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" ht="8" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="B6" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="C6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="D6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="E6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="F6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="G6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="I6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="K6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="M6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J2" s="3" t="s">
+      <c r="N6" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="C7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="J7" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="K7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
+      <c r="L7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
+      <c r="B8" s="7"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="7"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+      <c r="N8" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>